<commit_message>
feat: enhance backend features for generate subtask and integrate with telegram
</commit_message>
<xml_diff>
--- a/Members.xlsx
+++ b/Members.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E1C353-ACC0-4951-A650-D5FF4B540E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1678FE-F9D5-438B-84AE-9B69D557CD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8E26891F-89C6-4966-9756-B6289C2F9232}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Personal_Number</t>
   </si>
@@ -82,6 +82,12 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>Sukro</t>
+  </si>
+  <si>
+    <t>Mobile</t>
   </si>
 </sst>
 </file>
@@ -528,6 +534,17 @@
         <v>12</v>
       </c>
     </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>70004359</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+    </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F16" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
feat: enhance endpoint and result generate
</commit_message>
<xml_diff>
--- a/Members.xlsx
+++ b/Members.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A1678FE-F9D5-438B-84AE-9B69D557CD70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1A1C38-F14D-4168-8050-8CC52118F03C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8E26891F-89C6-4966-9756-B6289C2F9232}"/>
   </bookViews>
@@ -45,9 +45,6 @@
     <t>Role</t>
   </si>
   <si>
-    <t>Budi</t>
-  </si>
-  <si>
     <t>Danar</t>
   </si>
   <si>
@@ -88,6 +85,9 @@
   </si>
   <si>
     <t>Mobile</t>
+  </si>
+  <si>
+    <t>Muhammad Habibi</t>
   </si>
 </sst>
 </file>
@@ -443,6 +443,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.1796875" customWidth="1"/>
+    <col min="2" max="2" width="37.6328125" customWidth="1"/>
     <col min="3" max="3" width="13.6328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -462,10 +463,10 @@
         <v>70004353</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -473,10 +474,10 @@
         <v>70004354</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -484,10 +485,10 @@
         <v>70004352</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -495,10 +496,10 @@
         <v>70004355</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -506,10 +507,10 @@
         <v>70004356</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -517,10 +518,10 @@
         <v>70004357</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -528,10 +529,10 @@
         <v>70004358</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
@@ -539,15 +540,15 @@
         <v>70004359</v>
       </c>
       <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>16</v>
-      </c>
-      <c r="C9" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(subtasks): clean bracket prefixes and correct UI task role classification
</commit_message>
<xml_diff>
--- a/Members.xlsx
+++ b/Members.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F1A1C38-F14D-4168-8050-8CC52118F03C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35285735-5089-4BE2-A5DC-841B6188A4C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8E26891F-89C6-4966-9756-B6289C2F9232}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Personal_Number</t>
   </si>
@@ -48,33 +48,15 @@
     <t>Danar</t>
   </si>
   <si>
-    <t>Baril</t>
-  </si>
-  <si>
-    <t>Bone</t>
-  </si>
-  <si>
-    <t>Bukong</t>
-  </si>
-  <si>
     <t>Frontend</t>
   </si>
   <si>
     <t>Backend</t>
   </si>
   <si>
-    <t>QA Engineer</t>
-  </si>
-  <si>
-    <t>Project Officer</t>
-  </si>
-  <si>
     <t>SAD</t>
   </si>
   <si>
-    <t>Martin</t>
-  </si>
-  <si>
     <t>Marko</t>
   </si>
   <si>
@@ -88,6 +70,12 @@
   </si>
   <si>
     <t>Muhammad Habibi</t>
+  </si>
+  <si>
+    <t>Maulana Aryan</t>
+  </si>
+  <si>
+    <t>Sindu Sanova</t>
   </si>
 </sst>
 </file>
@@ -463,10 +451,10 @@
         <v>70004353</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
@@ -477,7 +465,7 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -485,10 +473,10 @@
         <v>70004352</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -496,10 +484,10 @@
         <v>70004355</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -507,10 +495,10 @@
         <v>70004356</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -518,37 +506,15 @@
         <v>70004357</v>
       </c>
       <c r="B7" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>70004358</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>70004359</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-    </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="F16" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>